<commit_message>
add dish 33 红烧冬瓜
</commit_message>
<xml_diff>
--- a/菜品数据.xlsx
+++ b/菜品数据.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1630,10 +1630,49 @@
 三、关键提示：内酯豆腐质地软嫩，烤后外焦里嫩，鸡蛋液增加风味层次；空气炸锅温度时间可依设备调整，避免烤糊；不吃辣可减少小米辣和辣椒面用量，喜酱香可加少许蚝油。</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>内酯豆腐1盒、鸡蛋1个、蒜末适量、小米辣适量、葱花适量、盐1勺、辣椒面1大勺、生抽1勺、老抽1勺、食用油适量</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>红烧冬瓜</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>正餐</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>素菜</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>冬瓜，大蒜</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>1.切冬瓜：尽量选黑皮冬瓜，皮切薄一点、多留厚的冬瓜皮肉，切成块后把瓤扔掉。
+2.锅中放足够多的水没过冬瓜块，同时放入两块大蒜头。
+3.放一个八角、一个桂皮、两勺生抽、一勺老抽、一点盐，再加冰糖、蚝油，最后放一点猪油（关键）。
+4.大火烧开后转中小火烧15到20分钟，把水尽量烧干，再加一点土豆粉或生粉勾芡。
+5.最后撒一点香葱出锅。</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>冬瓜1个、大蒜头2块、八角1个、桂皮1个、生抽2勺、老抽1勺、盐少许、冰糖适量、蚝油适量、猪油少许、土豆粉或生粉适量、香葱少许</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1956,7 +1995,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1975,7 +2014,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2029,7 +2068,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -2094,7 +2133,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2378,6 +2417,17 @@
       </c>
       <c r="H34">
         <f>COUNTIF(选菜记录!$D:$D,G34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>红烧冬瓜</t>
+        </is>
+      </c>
+      <c r="H35">
+        <f>COUNTIF(选菜记录!$D:$D,G35)</f>
         <v/>
       </c>
     </row>

</xml_diff>